<commit_message>
refactor(dongtan-tram): remove all VBA macro code and double-click hyperlink handlers from v8.xlsm
</commit_message>
<xml_diff>
--- a/01_전문업무_및_엔지니어링/11_현장_프로젝트/01_동탄트램/08.메뉴얼 및 평면도/최종/02_메뉴얼 공종프로섹스(집행단계)/매뉴얼 BODY (집행단계)v8.xlsx
+++ b/01_전문업무_및_엔지니어링/11_현장_프로젝트/01_동탄트램/08.메뉴얼 및 평면도/최종/02_메뉴얼 공종프로섹스(집행단계)/매뉴얼 BODY (집행단계)v8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sskjh\antigravity\01_전문업무_및_엔지니어링\11_현장_프로젝트\01_동탄트램\08.메뉴얼 및 평면도\최종\02_메뉴얼 공종프로섹스(집행단계)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5DBD876-39C2-4679-97B6-DA3F7FA4A645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEE9C214-AED6-466A-ADA5-E477AD29DB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="771" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12498,15 +12498,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -12515,17 +12524,8 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -12857,7 +12857,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="148" t="s">
+      <c r="B2" s="156" t="s">
         <v>575</v>
       </c>
       <c r="C2" s="149"/>
@@ -12878,58 +12878,58 @@
       </c>
     </row>
     <row r="6" spans="2:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="154" t="s">
+      <c r="B6" s="146" t="s">
         <v>577</v>
       </c>
       <c r="C6" s="147"/>
-      <c r="D6" s="154" t="s">
+      <c r="D6" s="146" t="s">
         <v>578</v>
       </c>
       <c r="E6" s="147"/>
-      <c r="F6" s="154" t="s">
+      <c r="F6" s="146" t="s">
         <v>579</v>
       </c>
       <c r="G6" s="147"/>
-      <c r="H6" s="154" t="s">
+      <c r="H6" s="146" t="s">
         <v>580</v>
       </c>
       <c r="I6" s="147"/>
-      <c r="J6" s="154" t="s">
+      <c r="J6" s="146" t="s">
         <v>581</v>
       </c>
       <c r="K6" s="147"/>
-      <c r="L6" s="154" t="s">
+      <c r="L6" s="146" t="s">
         <v>582</v>
       </c>
       <c r="M6" s="147"/>
     </row>
     <row r="7" spans="2:13" ht="28.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="152" t="str">
+      <c r="B7" s="155" t="str">
         <f>E21&amp;" 개"</f>
         <v>233 개</v>
       </c>
       <c r="C7" s="147"/>
-      <c r="D7" s="152" t="str">
+      <c r="D7" s="155" t="str">
         <f>F21&amp;" 개 (100%)"</f>
         <v>263 개 (100%)</v>
       </c>
       <c r="E7" s="147"/>
-      <c r="F7" s="152" t="str">
+      <c r="F7" s="155" t="str">
         <f>G21&amp;" 개 (100%)"</f>
         <v>263 개 (100%)</v>
       </c>
       <c r="G7" s="147"/>
-      <c r="H7" s="152" t="str">
+      <c r="H7" s="155" t="str">
         <f>H21&amp;" 개 (100%)"</f>
         <v>263 개 (100%)</v>
       </c>
       <c r="I7" s="147"/>
-      <c r="J7" s="152" t="str">
+      <c r="J7" s="155" t="str">
         <f>I21&amp;" 개 (100%)"</f>
         <v>233 개 (100%)</v>
       </c>
       <c r="K7" s="147"/>
-      <c r="L7" s="152" t="str">
+      <c r="L7" s="155" t="str">
         <f>J21&amp;" 개 (87.8%)"</f>
         <v>231 개 (87.8%)</v>
       </c>
@@ -13359,11 +13359,11 @@
       </c>
     </row>
     <row r="25" spans="2:12" ht="25.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="153" t="s">
+      <c r="B25" s="148" t="s">
         <v>610</v>
       </c>
       <c r="C25" s="147"/>
-      <c r="D25" s="153" t="s">
+      <c r="D25" s="148" t="s">
         <v>611</v>
       </c>
       <c r="E25" s="149"/>
@@ -13378,11 +13378,11 @@
       </c>
     </row>
     <row r="26" spans="2:12" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="156" t="s">
+      <c r="B26" s="152" t="s">
         <v>613</v>
       </c>
       <c r="C26" s="147"/>
-      <c r="D26" s="151" t="s">
+      <c r="D26" s="154" t="s">
         <v>614</v>
       </c>
       <c r="E26" s="149"/>
@@ -13397,11 +13397,11 @@
       </c>
     </row>
     <row r="27" spans="2:12" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B27" s="155" t="s">
+      <c r="B27" s="153" t="s">
         <v>616</v>
       </c>
       <c r="C27" s="147"/>
-      <c r="D27" s="150" t="s">
+      <c r="D27" s="151" t="s">
         <v>617</v>
       </c>
       <c r="E27" s="149"/>
@@ -13416,11 +13416,11 @@
       </c>
     </row>
     <row r="28" spans="2:12" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="156" t="s">
+      <c r="B28" s="152" t="s">
         <v>618</v>
       </c>
       <c r="C28" s="147"/>
-      <c r="D28" s="151" t="s">
+      <c r="D28" s="154" t="s">
         <v>619</v>
       </c>
       <c r="E28" s="149"/>
@@ -13435,11 +13435,11 @@
       </c>
     </row>
     <row r="29" spans="2:12" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B29" s="155" t="s">
+      <c r="B29" s="153" t="s">
         <v>620</v>
       </c>
       <c r="C29" s="147"/>
-      <c r="D29" s="150" t="s">
+      <c r="D29" s="151" t="s">
         <v>621</v>
       </c>
       <c r="E29" s="149"/>
@@ -13454,11 +13454,11 @@
       </c>
     </row>
     <row r="30" spans="2:12" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="156" t="s">
+      <c r="B30" s="152" t="s">
         <v>622</v>
       </c>
       <c r="C30" s="147"/>
-      <c r="D30" s="151" t="s">
+      <c r="D30" s="154" t="s">
         <v>623</v>
       </c>
       <c r="E30" s="149"/>
@@ -13481,11 +13481,11 @@
       <c r="B34" s="94" t="s">
         <v>585</v>
       </c>
-      <c r="C34" s="146" t="s">
+      <c r="C34" s="150" t="s">
         <v>625</v>
       </c>
       <c r="D34" s="147"/>
-      <c r="E34" s="146" t="s">
+      <c r="E34" s="150" t="s">
         <v>626</v>
       </c>
       <c r="F34" s="149"/>
@@ -13502,11 +13502,11 @@
       <c r="B35" s="93" t="s">
         <v>628</v>
       </c>
-      <c r="C35" s="155" t="s">
+      <c r="C35" s="153" t="s">
         <v>629</v>
       </c>
       <c r="D35" s="147"/>
-      <c r="E35" s="150" t="s">
+      <c r="E35" s="151" t="s">
         <v>630</v>
       </c>
       <c r="F35" s="149"/>
@@ -13523,11 +13523,11 @@
       <c r="B36" s="93" t="s">
         <v>632</v>
       </c>
-      <c r="C36" s="155" t="s">
+      <c r="C36" s="153" t="s">
         <v>633</v>
       </c>
       <c r="D36" s="147"/>
-      <c r="E36" s="150" t="s">
+      <c r="E36" s="151" t="s">
         <v>634</v>
       </c>
       <c r="F36" s="149"/>
@@ -13542,22 +13542,6 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="D25:K25"/>
-    <mergeCell ref="E34:K34"/>
-    <mergeCell ref="D29:K29"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="D28:K28"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:K30"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="E35:K35"/>
-    <mergeCell ref="C34:D34"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="E36:K36"/>
     <mergeCell ref="D26:K26"/>
@@ -13573,6 +13557,22 @@
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="D27:K27"/>
     <mergeCell ref="D7:E7"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="D28:K28"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:K30"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="E35:K35"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="D25:K25"/>
+    <mergeCell ref="E34:K34"/>
+    <mergeCell ref="D29:K29"/>
+    <mergeCell ref="B26:C26"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(mech): streamline purpose (Col J) and detail multi-step method (Col K) in machine excel sheet
</commit_message>
<xml_diff>
--- a/01_전문업무_및_엔지니어링/11_현장_프로젝트/01_동탄트램/08.메뉴얼 및 평면도/최종/02_메뉴얼 공종프로섹스(집행단계)/매뉴얼 BODY (집행단계)v8.xlsx
+++ b/01_전문업무_및_엔지니어링/11_현장_프로젝트/01_동탄트램/08.메뉴얼 및 평면도/최종/02_메뉴얼 공종프로섹스(집행단계)/매뉴얼 BODY (집행단계)v8.xlsx
@@ -10592,8 +10592,8 @@
     <col width="28" customWidth="1" style="147" min="7" max="7"/>
     <col width="12" customWidth="1" style="147" min="8" max="8"/>
     <col width="12" customWidth="1" style="147" min="9" max="9"/>
-    <col width="36" customWidth="1" style="147" min="10" max="10"/>
-    <col width="32" customWidth="1" style="147" min="11" max="11"/>
+    <col width="38" customWidth="1" style="147" min="10" max="10"/>
+    <col width="52" customWidth="1" style="147" min="11" max="11"/>
     <col width="28" customWidth="1" style="147" min="12" max="12"/>
     <col width="36" customWidth="1" style="147" min="13" max="13"/>
     <col width="24" customWidth="1" style="147" min="14" max="14"/>
@@ -10719,7 +10719,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" s="147">
+    <row r="2" ht="48" customHeight="1" s="147">
       <c r="A2" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -10767,12 +10767,14 @@
       </c>
       <c r="J2" s="156" t="inlineStr">
         <is>
-          <t>동탄도시철도(트램) 기계설비(HVAC, 급배수, 위생, 오폐수, 승강기) 및 소방설비(소화, 제연, 경보)의 착공 전 설계도서(도면·시방서·수량산출서·내역서)의 적격성을 검토하고, 지하 및 지상 정거장, 변전소, 차량기지 내 법적 기준 충족 및 시공성을 사전 확보한다.</t>
+          <t>기계·소방설비 설계도서(도면/시방/계산서)의 KDS 47 및 NFTC 기준 적합성과 시공성·경제성 사전 검증</t>
         </is>
       </c>
       <c r="K2" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 설계도서 및 계산서 총괄 수집, STEP 2: 삼각 교차 대조 및 물량 정합성 검증 절차서 준수 시공</t>
+          <t>1) STEP 1 (설계도서 삼각 대조): KDS 47/NFTC 기준에 따라 공조/환기 부하계산서, 설계도면, 수량산출서 1:1 정합성 검증
+2) STEP 2 (주요 장비 용량 검토): 변전소 PAC(3대), 고내열 제연팬(250℃/1h), 인버터 펌프 정격 양정/유량 시방 일치성 확인
+3) STEP 3 (인터페이스 및 개선안 도출): 건축 슬리브, 전기 NFR-8 내화배선, 신호 배수공동구 연계성 검토 및 설계변경안 감리 승인</t>
         </is>
       </c>
       <c r="L2" s="156" t="inlineStr">
@@ -10831,7 +10833,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" s="147">
+    <row r="3" ht="48" customHeight="1" s="147">
       <c r="A3" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -10879,12 +10881,14 @@
       </c>
       <c r="J3" s="163" t="inlineStr">
         <is>
-          <t>기계 및 소방공사의 성공적인 수행을 위해 발주처, 책임감리단, 원도급사, 전문협력업체가 참여하는 Kick-Off Meeting을 개최하여 중점 품질관리 항목, 법적 인허가 일정, 장비 제작납기 및 자재 승인 프로세스를 일괄 확정한다.</t>
+          <t>기계·소방 공종 3자(발주처-감리-시공) 킥오프를 통한 주요 자재 조달 라인 및 4대 공정 마일스톤 확정</t>
         </is>
       </c>
       <c r="K3" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: KOM 킥오프 회의 소집 및 R&amp;R 확정, STEP 2: 주요 장비 제작 및 조달 계획 수립 절차서 준수 시공</t>
+          <t>1) STEP 1 (3자 협의체 구성): 발주처, 책임감리단, 기계/소방 협력사 간 공정·품질·안전 관리체계 및 업무 R&amp;R 확정
+2) STEP 2 (주요 자재 수급선 검토): STS 강관, 덕트, 펌프, 승강기 등 장납기 자재의 공장 승인 및 납품 스케줄 동기화
+3) STEP 3 (핵심 마일스톤 수립): 3D BIM 간섭해소, FAT 공장검수, 수압시험, 소방 완공검사 등 공정 임계경로(CP) 관리</t>
         </is>
       </c>
       <c r="L3" s="163" t="inlineStr">
@@ -10943,7 +10947,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" s="147">
+    <row r="4" ht="48" customHeight="1" s="147">
       <c r="A4" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -10991,12 +10995,14 @@
       </c>
       <c r="J4" s="156" t="inlineStr">
         <is>
-          <t>지하 정거장 천장 및 기계실, 차량기지 검수고 등 배관·덕트 밀집 구역에 대해 3D BIM(LOD 350) 통합 모델링을 수행하여 타 공종(건축, 전기, 신호, 궤도)과의 물리적 간섭을 착공 전 100% 제거하고 최적의 시공 동선을 도출한다.</t>
+          <t>LOD 350 기반 3D BIM을 활용하여 기계덕트·소화배관·전기트레이 간 Hard Clash 0건 달성 및 CSD 승인</t>
         </is>
       </c>
       <c r="K4" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 3D BIM 기계/소방 상세 모델링 (LOD 350), STEP 2: 다공종 통합 모델 합성 및 간섭 체크 절차서 준수 시공</t>
+          <t>1) STEP 1 (LOD 350 3D 모델링): 기계 공조덕트, 소화배관, 위생배관 및 전기 트레이의 3D 통합 모델 구축
+2) STEP 2 (복합 간섭체크 실행): Navisworks 간섭 체크 엔진을 가동하여 배관 교차 및 건축 골조 간섭(Clash) 전수 색출
+3) STEP 3 (시공상세도 CSD 확정): 정거장 유효 천장고(CH ≥ 2.7m) 확보를 위한 배관 입체 재배치 및 감리단 CSD 최종 승인</t>
         </is>
       </c>
       <c r="L4" s="156" t="inlineStr">
@@ -11055,7 +11061,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" s="147">
+    <row r="5" ht="48" customHeight="1" s="147">
       <c r="A5" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11103,12 +11109,14 @@
       </c>
       <c r="J5" s="163" t="inlineStr">
         <is>
-          <t>소방시설공사업법 및 물환경보전법에 따라 공사 착공 전 관할 소방서로부터 소방시설 시공 동의 및 착공신고를 득하고, 차량기지 위험물 저장소, 비상발전기 유류탱크, 오수처리시설 인허가를 적기에 완료하여 법적 리스크를 제거한다.</t>
+          <t>소방시설공사업법 제13조에 따른 착공신고 및 위험물·오폐수 환경 인허가 적기 득</t>
         </is>
       </c>
       <c r="K5" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 소방시설 착공신고서 작성 및 도서 구비, STEP 2: 소방시설 건축동의 및 기술 검토 보완 절차서 준수 시공</t>
+          <t>1) STEP 1 (소방 착공신고): 소방기술자/감리원 배치신고서 및 소방 설계도서를 관할 화성소방서에 제출하여 착공필증 수령
+2) STEP 2 (위험물 저장 승인): 비상발전기 유류탱크(경유) 저장소 설치허가 및 방유제(용량 110%) 안전기준 검증
+3) STEP 3 (환경 인허가 완료): 차량기지 오폐수배출시설 설치신고 및 수질 TMS 연동 계획 관할 지자체 승인</t>
         </is>
       </c>
       <c r="L5" s="163" t="inlineStr">
@@ -11167,7 +11175,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" s="147">
+    <row r="6" ht="48" customHeight="1" s="147">
       <c r="A6" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11215,12 +11223,14 @@
       </c>
       <c r="J6" s="156" t="inlineStr">
         <is>
-          <t>지하 정거장 기계실 및 차량기지 종합검수동에 설치되는 대형 중량물(공기조화기, 냉동기, 소방펌프, 열교환기)의 반입 개구부, 수직 인양 동선, 양중 크레인 작업 반경 및 현장 자재 야적장 보관 관리 계획을 수립한다.</t>
+          <t>지하 기계실 대형 장비(AHU, 펌프 등)의 DA 개구부 양중 및 안전 반입 동선 확보</t>
         </is>
       </c>
       <c r="K6" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 중량 장비 제원 및 반입 경로 실측, STEP 2: 양중 크레인 작업 계획 및 안전성 검토 절차서 준수 시공</t>
+          <t>1) STEP 1 (양중 크레인 계획): 50ton 하이드로 크레인 작업반경 설정, 복공판 하부 지지력(K30 ≥ 150) 및 아웃트리거 보강
+2) STEP 2 (개구부 통과 검토): 장비 분할 치수와 DA 개구부(W2.5m x L4.0m) 유효 통과폭 대조 및 호이스트/체인블록 가설
+3) STEP 3 (수평 인입 및 안착): 운반 롤러 및 레일 시스템을 이용하여 기계실 기초 패드 위로 유도 후 레벨링 및 앵커링</t>
         </is>
       </c>
       <c r="L6" s="156" t="inlineStr">
@@ -11279,7 +11289,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" s="147">
+    <row r="7" ht="48" customHeight="1" s="147">
       <c r="A7" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11327,12 +11337,14 @@
       </c>
       <c r="J7" s="163" t="inlineStr">
         <is>
-          <t>동탄트램 복합 공정의 성공을 위해 기계·소방 분야와 6대 연관 공종(토목 노반, 궤도 콘크리트도상, 건축 구조/마감, 전기 수변전, 신호 연동, 통신 LTE-R) 간의 주간 Big Room 합동 회의를 운영하여 시공 오차 및 인터페이스 누락을 원천 차단한다.</t>
+          <t>건축, 전기, 통신, 신호, 궤도 등 타 공종과의 시공 간섭 배제 및 시공 우선순위 룰 확립</t>
         </is>
       </c>
       <c r="K7" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: Big Room 합동 회의 안건 도출 및 3D 모델 준비, STEP 2: 7대 공종 합동 기술 조율 및 대안 확정 절차서 준수 시공</t>
+          <t>1) STEP 1 (Big Room 정례협의): 7대 공종 합동 주간 인터페이스 회의를 운영하여 주배관과 타 공종 지장물 간섭 해소
+2) STEP 2 (시공 우선순위 확정): 슬리브 선매립(건축) ⟶ 대형 풍도/주배관(기계) ⟶ 케이블트레이(전기) 순차 시공 룰 적용
+3) STEP 3 (인터페이스 체크시트 발행): 상호 인계인수 전 슬리브 위치, 방화구획, 배수구 트렌치 시공 상태 합동 서명 검측</t>
         </is>
       </c>
       <c r="L7" s="163" t="inlineStr">
@@ -11391,7 +11403,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" s="147">
+    <row r="8" ht="48" customHeight="1" s="147">
       <c r="A8" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11439,12 +11451,14 @@
       </c>
       <c r="J8" s="156" t="inlineStr">
         <is>
-          <t>트램 본선 도로 하부 및 정거장 외부 인입 구역에 매설되는 기계배관(상수도 급수관, 지열 집열관, 오배수 연결관)에 대해 지자체(화성시), 도로관리청 및 한국전력·가스·통신 유관기관과 지장물 이설 및 도로굴착 점용 협의를 수행한다.</t>
+          <t>트램 본선 도로 하부 지중매설 배관(상수도, 지열, 우오수)과 지하 지장물 간 안전 이격거리 확보</t>
         </is>
       </c>
       <c r="K8" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 지하 지장물 매설도 수집 및 3D GPR 탐사, STEP 2: 유관기관 협의 및 도로굴착점용 허가 획득 절차서 준수 시공</t>
+          <t>1) STEP 1 (3D 지하매설물 탐사): GPR 탐사 및 줄파기를 통해 기존 가스관, 한전관로, 통신관로 심도와 좌표 정밀 확인
+2) STEP 2 (안전 이격거리 유지): 타 지장물과 최소 300mm 이상 이격 배치하고 고저차 간섭 시 강관 보호공(Casing) 적용
+3) STEP 3 (모래부설 및 다짐): 배관 주위 양질의 모래(두께 100mm) 부설 후 되메우기 층별 다짐(다짐도 ≥ 95%) 및 경고테이프 매설</t>
         </is>
       </c>
       <c r="L8" s="156" t="inlineStr">
@@ -11503,7 +11517,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" s="147">
+    <row r="9" ht="48" customHeight="1" s="147">
       <c r="A9" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11551,12 +11565,14 @@
       </c>
       <c r="J9" s="163" t="inlineStr">
         <is>
-          <t>KCS 41(건축기계설비공사 표준시방서) 및 KDS 47(철도설계기준)에 의거하여 기계·소방설비의 단계별 세부 시공 방법, 동원 인원 및 장비 계획, 용접 절차서(WPS), 비파괴검사(NDT), 수압시험 및 품질·안전관리 종합 시공계획서를 작성하여 감리단 승인을 득한다.</t>
+          <t>KCS 41 시방 기준 준수, 유자격 용접사 WPS 승인 및 밀폐공간 안전보건 체계 확립</t>
         </is>
       </c>
       <c r="K9" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 공종별 세부 시공 방법 및 절차서 작성, STEP 2: 자재 시험 및 품질관리 계획서 수립 절차서 준수 시공</t>
+          <t>1) STEP 1 (공종별 절차서 수립): 배관, 덕트, 장비설치 등 세부 작업별 인원·장비·공정 계획 및 위험성평가서 작성
+2) STEP 2 (WPS 용접절차 승인): 배관 재질별(STS, 탄소강) 용접절차시방서(WPS) 수립 및 유자격 용접사 시험편 PQR 검증
+3) STEP 3 (밀폐공간 안전관리): 지하 집수조/탱크 작업 시 복합가스(산소, 황화수소) 측정, 송기마스크 착용 및 감시원 상주</t>
         </is>
       </c>
       <c r="L9" s="163" t="inlineStr">
@@ -11615,7 +11631,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1" s="147">
+    <row r="10" ht="48" customHeight="1" s="147">
       <c r="A10" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11663,12 +11679,14 @@
       </c>
       <c r="J10" s="156" t="inlineStr">
         <is>
-          <t>현장에 반입되는 배관용 스테인리스 강관, 인버터 가압 부스터펌프, 옥내소화전함, 밸브류, 공조기 등 주요 기자재에 대해 KS 인증서, 공인기관 시험성적서(밀시트), 공장검수(FAT) 성적을 1:1 대조하여 불량 자재의 현장 반입을 원천 차단한다.</t>
+          <t>배관, 밸브, 펌프 등 주요 기계·소방 기자재의 KS/KFI 규격 검증 및 공장 시험(FAT) 수행</t>
         </is>
       </c>
       <c r="K10" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 자재 공급원 승인 요청서(MAR) 접수 및 검토, STEP 2: 주요 대형 장비 공장검수(FAT) 수행 절차서 준수 시공</t>
+          <t>1) STEP 1 (공장검수 FAT 실시): 인버터 부스터펌프, 공조기 공장을 방문하여 모터 효율, 정격 양정·유량, 소음·진동 시험 입회
+2) STEP 2 (자재 현장 반입 검수): 밀시트(Mill Sheet), KS/KFI 인증서 확인 및 STS 강관 두께·진원도 마이크로미터 정밀 검측
+3) STEP 3 (자재 보관 및 불합격 통제): 배관 단부 보호캡 체결, 옥내 전용 적치장 보관 및 불합격 자재 24시간 이내 반출 조치</t>
         </is>
       </c>
       <c r="L10" s="156" t="inlineStr">
@@ -11727,7 +11745,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1" s="147">
+    <row r="11" ht="48" customHeight="1" s="147">
       <c r="A11" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11775,12 +11793,14 @@
       </c>
       <c r="J11" s="163" t="inlineStr">
         <is>
-          <t>건축물의 피난·방화구조 등의 기준에 관한 규칙에 따라 방화벽, 바닥 슬래브를 관통하는 기계 배관, 냉매관, 공조 덕트 주변의 관통 틈새에 대해 화재안전연구원 공인 인증을 득한 내화채움재(내화패드, 방화실란트, 차염/차열재)를 100% 밀폐 시공하여 화염 및 유독가스 층간 전파를 원천 차단한다.</t>
+          <t>콘크리트 골조 타설 전 관통 슬리브 선매립 및 2시간 차열·차염 내화채움구조 시공</t>
         </is>
       </c>
       <c r="K11" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 관통부 틈새 청소 및 공인 내화구조 매핑, STEP 2: 내부 불연재(미네랄울) 고밀도 충진 절차서 준수 시공</t>
+          <t>1) STEP 1 (골조 슬리브 선매립): 구조체 철근 배근 시 배관경 대비 1~2규격 큰 강관/PVC 슬리브 설치 및 단단히 고정
+2) STEP 2 (관통 틈새 내화충진): 배관 설치 후 슬리브 틈새에 고밀도 미네랄울(밀도 ≥ 100kg/㎥) 충진 및 방화실란트 15mm 도포
+3) STEP 3 (내화성능 확인): 공인기관 2시간 차열·차염 성적서 확인 및 우레탄폼 등 가연성 자재 사용 전면 금지 검측</t>
         </is>
       </c>
       <c r="L11" s="163" t="inlineStr">
@@ -11839,7 +11859,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1" s="147">
+    <row r="12" ht="48" customHeight="1" s="147">
       <c r="A12" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11887,12 +11907,14 @@
       </c>
       <c r="J12" s="156" t="inlineStr">
         <is>
-          <t>트램 본선 궤도 분기부 및 차량기지 내 총 143개소의 핵심 선로전환기(Point Machine)와 열차 위치 검지용 차축검지기(Axle Counter) 구역의 침수 불량 및 동절기 결빙 사고를 원천 방지하기 위하여 궤도 콘크리트 타설 전 하부 횡단 배수용 파이프 및 전선관로 공동구를 정밀 선시공한다.</t>
+          <t>본선 및 차량기지 143개소 선로전환기 하부 배수관로 선시공으로 동절기 결빙 및 침수 방지</t>
         </is>
       </c>
       <c r="K12" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 신호·궤도팀 합동 분기기 143개소 좌표 실측, STEP 2: 횡단 배수관로 매설 및 지지틀 고정 절차서 준수 시공</t>
+          <t>1) STEP 1 (드레인 피트 가설): 선로전환기 구동부 하부에 침전 드레인 피트 및 STS 타공 스트레이너 설치
+2) STEP 2 (횡단 배수관로 연결): 도상 횡단 배수관(D100/150)을 자연유하 구배(i ≥ 1.0%)로 선로변 주 집수정까지 직결
+3) STEP 3 (궤도 타설 전 통수시험): 궤도 콘크리트 타설 전 통수 및 수압시험을 실시하여 관로 막힘 및 누수 0건 최종 확인</t>
         </is>
       </c>
       <c r="L12" s="156" t="inlineStr">
@@ -11951,7 +11973,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1" s="147">
+    <row r="13" ht="48" customHeight="1" s="147">
       <c r="A13" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -11999,12 +12021,14 @@
       </c>
       <c r="J13" s="163" t="inlineStr">
         <is>
-          <t>화재안전기술기준(NFTC) 및 전기설비기술기준에 따라 소방펌프실 주펌프, 충압펌프, 지하차도 및 역사 제연팬에 공급되는 비상 전원 간선에 대해 최고 수준의 고내열 내화성능을 갖춘 NFR-8(또는 F-FR-8) 내화케이블을 전용 배관으로 포설하고, 전기분야 비상발전기·MCC반과 무결점 인터페이스를 완료한다.</t>
+          <t>소방펌프, 제연팬 등 소방설비의 10초 이내 비상전원 절환 및 NFR-8 내화배선 무중단 공급</t>
         </is>
       </c>
       <c r="K13" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 소방 기계 부하 용량(kW) 산정 및 전기팀 통보, STEP 2: NFR-8 고내열 내화케이블 전용 관로 시공 절차서 준수 시공</t>
+          <t>1) STEP 1 (비상전원 ATS 연계): 상용전원 정전 시 10초 이내 비상발전기 전원으로 자동 절환되는 ATS 인터록 구축
+2) STEP 2 (NFR-8 내화케이블 포설): 소방용 동력 간선에 고내열 NFR-8 케이블을 전용 금속관에 단독 배선하여 850℃ 내열 확보
+3) STEP 3 (MCC 제어반 세팅): 소방펌프 전용 MCC 제어반의 과부하 트립 기능을 배제(경보만 발생)하여 화재 시 연속 가동 보장</t>
         </is>
       </c>
       <c r="L13" s="163" t="inlineStr">
@@ -12063,7 +12087,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1" s="147">
+    <row r="14" ht="48" customHeight="1" s="147">
       <c r="A14" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -12111,12 +12135,14 @@
       </c>
       <c r="J14" s="156" t="inlineStr">
         <is>
-          <t>정거장 및 차량기지 지하 저수조 내에서 생활위생용수와 소화용수가 장기간 정체되어 발생하는 사수(死水, 물고임 부패) 현상을 방지하기 위하여, 급수펌프 흡입배관의 최저점을 소화용수 유효수위 상향으로 확보하고, 저수조 내부에 유지관리용 칸막이 1개소를 설치하는 고도화 수배관 시스템을 시공한다.</t>
+          <t>위생적인 STS304 패널형 저수조 설치, 생활용수 사수 방지 배관 및 소화수 유효용량 상시 확보</t>
         </is>
       </c>
       <c r="K14" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 저수조 용량 및 소화수 유효수위 계산, STEP 2: STS 패널형 저수조 조립 및 칸막이 가설 절차서 준수 시공</t>
+          <t>1) STEP 1 (STS 패널 조립 용접): STS304 패널 아르곤(TIG) 용접 조립 후 액체침투탐상(PT)으로 용접부 결함 100% 색출
+2) STEP 2 (사수방지 흡입배관 분리): 급수펌프 흡입관은 소화수위 상단에, 소방펌프 흡입관은 바닥 최하단에 분리 배치
+3) STEP 3 (만수 수밀시험): 저수조 만수 후 24시간 동안 수위 강하 및 외부 누수 유무를 정밀 측정하여 감리단 합격 승인</t>
         </is>
       </c>
       <c r="L14" s="156" t="inlineStr">
@@ -12175,7 +12201,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" s="147">
+    <row r="15" ht="48" customHeight="1" s="147">
       <c r="A15" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -12223,12 +12249,14 @@
       </c>
       <c r="J15" s="163" t="inlineStr">
         <is>
-          <t>신에너지 및 재생에너지 개발·이용·보급 촉진법 및 친환경 녹색건축물 인증 기준에 따라 차량기지 및 정거장에 지중 열교환용 고밀도 폴리에틸렌관(HDPE, KSM 3408)을 지하 150~200m 깊이로 천공 매설하고, 전기융착(EF) 접합 및 1.0MPa 수압시험, 친환경 벤토나이트 그라우팅을 완벽 시공한다.</t>
+          <t>수직 밀폐형 지열 U-Tube(심도 150m) 시공 및 친환경 지열 히트펌프 연계 열교환 극대화</t>
         </is>
       </c>
       <c r="K15" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 지열 천공 지점 측량 및 천공기 가설, STEP 2: U-Tube PE 열교환관 조립 및 1차 수압시험 절차서 준수 시공</t>
+          <t>1) STEP 1 (천공 및 U-Tube 삽입): 직경 150mm x 심도 150m 천공 후 고밀도 PE 파이프(KSM 3408, SDR11) U-Tube 삽입
+2) STEP 2 (열전도 그라우팅): 천공 하부부터 지표면까지 벤토나이트 혼합 그라우트재(열전도도 ≥ 1.8 W/m·K)를 가압 연속 주입
+3) STEP 3 (수압시험 및 헤더 연결): 1.0 MPa 수압으로 2시간 동안 압력 유지 확인 후 기계실 지열 헤더 매니폴드 연결</t>
         </is>
       </c>
       <c r="L15" s="163" t="inlineStr">
@@ -12287,7 +12315,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1" s="147">
+    <row r="16" ht="48" customHeight="1" s="147">
       <c r="A16" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -12335,12 +12363,14 @@
       </c>
       <c r="J16" s="156" t="inlineStr">
         <is>
-          <t>지하 정거장 대합실/승강장 및 변전실·전기실의 쾌적한 실내 환경 유지와 전기기기 발열 배출을 위해 KCS 41 시방서에 맞춰 아연도금강판(GI) 공조덕트를 시공하며, 변전실 시간당 10회 환기, 화장실 15~20회 음압 배기 및 동절기 외기 역류 방지용 B.D.D(기류역류방지댐퍼)를 완벽 가설한다.</t>
+          <t>변전실 1종 급기가압(10회/h, 실온 ≤40℃) 및 화장실 3종 음압 환기, 역류방지(B.D.D) 구축</t>
         </is>
       </c>
       <c r="K16" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 덕트 제작 치수 검수 및 아연도금강판 가공, STEP 2: 풍도 댐퍼 및 B.D.D 기류역류방지댐퍼 조립 절차서 준수 시공</t>
+          <t>1) STEP 1 (아연도강판 덕트 제작): KCS 41 시방 기준에 따라 아연도강판(GI) 피츠버그 록 성형 및 기밀 실링 시공
+2) STEP 2 (방진행거 및 댐퍼 취부): 덕트 하중 지지를 위한 방진스프링 행거(간격 ≤ 2.0m) 및 역류방지 댐퍼(B.D.D) 체결
+3) STEP 3 (덕트 누기시험): 연기발생기 및 차압계를 이용하여 허용 누기량(클래스 3 이하) 만족 여부 정밀 측정</t>
         </is>
       </c>
       <c r="L16" s="156" t="inlineStr">
@@ -12399,7 +12429,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1" s="147">
+    <row r="17" ht="48" customHeight="1" s="147">
       <c r="A17" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -12447,12 +12477,14 @@
       </c>
       <c r="J17" s="163" t="inlineStr">
         <is>
-          <t>도시철도건설규칙 및 화재안전기준(NFTC 501)에 따라 화재 시 발생하는 고온의 유독가스를 신속히 배출하기 위해, 250℃ 고온에서 1시간 이상 연속 운전이 가능한 공인 시험기관 인증 제연팬(Axial Fan), 내화 풍도, 1.5mm 아연도 강판 덕트 및 불연 내열 캔버스를 완벽 시공한다.</t>
+          <t>KFI 공인 250℃ 1시간 연속운전 고내열 제연팬 및 1.5mm 내화풍도 시공으로 화재 유독가스 배출</t>
         </is>
       </c>
       <c r="K17" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 250℃ 고내열 제연팬 사양 검토 및 반입 검수, STEP 2: 1.5mm 이상 고강도 제연 풍도 및 내진 지지대 시공 절차서 준수 시공</t>
+          <t>1) STEP 1 (고내열 제연팬 거치): KFI 250℃/1h 내열인증 H종 절연 제연팬을 방진 스프링 베이스 위에 수평 거치
+2) STEP 2 (내화 제연덕트 체결): 1.5mm 이상 두꺼운 강판 덕트에 1,000℃ 세라믹 불연 가스켓을 삽입하여 고장력 볼트 체결
+3) STEP 3 (내진 브레이싱 및 기동 시험): 종·횡방향 내진 버팀대(간격 9m/4.5m) 시공 후 화재 신호 수신 시 30초 내 기동 검증</t>
         </is>
       </c>
       <c r="L17" s="163" t="inlineStr">
@@ -12511,7 +12543,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1" s="147">
+    <row r="18" ht="48" customHeight="1" s="147">
       <c r="A18" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -12559,12 +12591,14 @@
       </c>
       <c r="J18" s="156" t="inlineStr">
         <is>
-          <t>차량기지 종합검수고동 등 층고가 높고 체적이 거대한 대공간을 전면 냉난방하는 에너지 비효율성을 방지하기 위하여, 정비원이 실제 작업하는 핏트(Pit) 및 차체 검수 구역에 이동식 에어컨과 원적외선 전기히터를 국부 배치하고, 변전소 전기실에는 패키지 에어컨(PAC)을 정밀 가설한다.</t>
+          <t>대공간 검수고 작업자 중심 국부 냉난방(이동식 에어컨/원적외선) 및 변전소 전용 PAC 3대 배치</t>
         </is>
       </c>
       <c r="K18" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 대공간 국부 작업 구역 부하 분석 및 장비 선정, STEP 2: 변전실 패키지 에어컨(PAC) 3대 정합성 가설 절차서 준수 시공</t>
+          <t>1) STEP 1 (변전소 PAC 3대 설치): 변전소별 패키지 에어컨(PAC) 3대를 등간격 배치하고 R-410A 냉매배관 기밀시험(3.8MPa)
+2) STEP 2 (검수고 국부 냉난방 가설): 정비 피트 및 작업대 위치에 이동식 플렉시블 토출 에어컨과 고효율 원적외선 난방기 설치
+3) STEP 3 (시운전 및 온습도 측정): 실별 자동온도조절기(TC) 세팅 및 24시간 연속 운전을 통해 실온 ≤ 28℃ 유지 성능 검증</t>
         </is>
       </c>
       <c r="L18" s="156" t="inlineStr">
@@ -12623,7 +12657,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1" s="147">
+    <row r="19" ht="48" customHeight="1" s="147">
       <c r="A19" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -12671,12 +12705,14 @@
       </c>
       <c r="J19" s="163" t="inlineStr">
         <is>
-          <t>중앙 기계실 냉동기, 열교환기, 펌프와 공조기를 연결하는 냉온수 및 냉각수 주배관에 대해 KCS 41 시방 기준에 따라 숙련된 유자격 용접사가 맞대기 아크용접 및 TIG 용접을 수행하고, 용접부 비파괴검사(RT ≥ 10%), 설계압력 1.5배 수압시험, 방청 도장 및 보온 단열재를 완벽 시공한다.</t>
+          <t>KSD 3562 탄소강관 맞대기 용접, 비파괴검사(RT ≥ 10%) 및 1.5MPa 수압시험을 통한 누수 Zero</t>
         </is>
       </c>
       <c r="K19" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 배관 절단 및 개선(Beveling) 가공, STEP 2: 가접 및 다층 맞대기 용접(WPS 준수) 절차서 준수 시공</t>
+          <t>1) STEP 1 (그루브 가공 및 맞대기 용접): 배관 단부 30~35° 베벨 가공 후 TIG 루트패스 및 아크 다층 맞대기 용접
+2) STEP 2 (방사선 비파괴검사 RT): 용접부의 10% 이상을 무작위 추출하여 방사선 투과 촬영(RT) 및 결함(기공, 슬래그) 100% 판독
+3) STEP 3 (1.5배 수압시험 및 보온): 설계압력 1.5배(1.5MPa) 60분 무누수 확인 후 난연 고무발포 단열재(40mm) 밀착 시공</t>
         </is>
       </c>
       <c r="L19" s="163" t="inlineStr">
@@ -12735,7 +12771,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1" s="147">
+    <row r="20" ht="48" customHeight="1" s="147">
       <c r="A20" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -12783,12 +12819,14 @@
       </c>
       <c r="J20" s="156" t="inlineStr">
         <is>
-          <t>도시철도건설규칙 제67조에 따라 능동지하차도 트램 전용터널 통과 구간에 화재 발생 시 승객의 안전 피난 방향으로 연기 유동을 제어(임계풍속 ≥ 2.5m/s 확보)하는 제연설비, 건식 연결송수관 및 CFD 컴퓨터 화재 수치해석 시뮬레이션을 완벽 시공·검증한다.</t>
+          <t>지하차도 트램 전용터널 제연(Jet Fan 임계풍속 ≥ 2.5m/s) 및 50m 간격 건식 연결송수관 구축</t>
         </is>
       </c>
       <c r="K20" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 3D CFD 화재 및 피난 시뮬레이션 모델링, STEP 2: 터널 천장 제연팬(Jet Fan) 앵커링 및 내진 시공 절차서 준수 시공</t>
+          <t>1) STEP 1 (Jet Fan 천장 앵커링): 터널 천장부에 진동 감쇠 방진행거 및 고장력 케미컬 앵커로 Jet Fan 안전 체결
+2) STEP 2 (3D CFD 풍속 검증): 터널 화재 시뮬레이션 기반 임계풍속(2.5m/s) 도출 및 연기 역류(Backlayering) 차단 검증
+3) STEP 3 (건식 연결송수관 시공): 50m 간격 방수구함(D100 Sch40) 설치 및 2.0MPa 고압 수압시험을 통한 배관 내력 확인</t>
         </is>
       </c>
       <c r="L20" s="156" t="inlineStr">
@@ -12847,7 +12885,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1" s="147">
+    <row r="21" ht="48" customHeight="1" s="147">
       <c r="A21" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -12895,12 +12933,14 @@
       </c>
       <c r="J21" s="163" t="inlineStr">
         <is>
-          <t>지하 정거장 공조기계실 및 전기실에 대형 공기조화기(AHU)와 항온항습기(PAC)를 반입하여 기초 콘크리트 패드 위에 거치하고, 기계 가동 진동이 건축 구조물로 전파되는 것을 차단하는 방진스프링 마운트(정적변위 25~50mm), 드레인 트랩 및 수평도(±1mm)를 완벽 시공한다.</t>
+          <t>공조기 케이싱 수평 거치, 방진마운트(정적변위 ≥ 25mm) 진동 차단 및 딥 U-Trap 배수</t>
         </is>
       </c>
       <c r="K21" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 기초 콘크리트 패드 검측 및 기준선 마킹, STEP 2: AHU 분할 반입 및 블록 조립 결속 절차서 준수 시공</t>
+          <t>1) STEP 1 (기초 패드 및 방진마운트): 콘크리트 패드 위에 정적 변위 25mm 밀폐형 스프링 방진기 설치 및 수평 레벨링
+2) STEP 2 (불연 캔버스 연결): 송풍기 토출구와 덕트 사이에 실리콘 코팅 불연 캔버스를 주름 없이 견고히 체결
+3) STEP 3 (딥 U-Trap 드레인 시공): 흡입 부압에 견디도록 유효 봉수 100mm 이상의 드레인 트랩 시공 후 배수 통수시험</t>
         </is>
       </c>
       <c r="L21" s="163" t="inlineStr">
@@ -12959,7 +12999,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1" s="147">
+    <row r="22" ht="48" customHeight="1" s="147">
       <c r="A22" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13007,12 +13047,14 @@
       </c>
       <c r="J22" s="156" t="inlineStr">
         <is>
-          <t>정거장 및 차량기지 관리동의 위생적인 음용수 및 급탕 공급을 위하여 KSD 3595(일반배관용 스테인리스 강관) 및 KSD 3576(배관용 스테인리스 강관)을 적용하고, 전용 전동 압착공구를 사용한 무용접 프레스 조인트 시공, 1.0MPa 수압시험, 배관 내부 염소 소독 세척을 완벽 수행한다.</t>
+          <t>STS304 강관 무용접 프레스 피팅 전동 압착, 1.0MPa 수압시험 및 위생 염소소독 완료</t>
         </is>
       </c>
       <c r="K22" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: STS 파이프 정밀 절단 및 단부 버(Burr) 제거, STEP 2: 피팅 삽입 깊이 마킹 및 전동 압착 체결 절차서 준수 시공</t>
+          <t>1) STEP 1 (관 절단 및 프레스 압착): 롤러 커터로 관 직각 절단, 리머 버 제거, EPDM 오링 삽입 후 전동 압착공구 체결
+2) STEP 2 (육각 게이지 전수 검측): 전용 판정 게이지(Go/No-Go)를 결합부에 밀착하여 압착 치수 정밀도 100% 전수 검사
+3) STEP 3 (수압시험 및 차아염소산 소독): 1.0MPa 60분 수압 무누수 확인 후 50ppm 염소수로 24시간 통수 살균 및 수질검사</t>
         </is>
       </c>
       <c r="L22" s="156" t="inlineStr">
@@ -13071,7 +13113,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1" s="147">
+    <row r="23" ht="48" customHeight="1" s="147">
       <c r="A23" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13119,12 +13161,14 @@
       </c>
       <c r="J23" s="163" t="inlineStr">
         <is>
-          <t>정거장 화장실 오수, 바닥 잡배수 및 지하 침출수를 신속하고 안전하게 배출하기 위해, 오배수 배관의 자연유하 구배(1/50~1/100)를 확보하고, 지하 최하층 집수조에 고효율 수중 카터/오수 배수펌프 2대(1대 상용, 1대 예비)와 수위센서 연동 자동 교번 운전 제어반을 완벽 시공한다.</t>
+          <t>오배수관 자연유하 구배(i ≥ 1/100) 유지 및 집수조 수중배수펌프 자동교번 4단 수위제어</t>
         </is>
       </c>
       <c r="K23" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 오배수 배관 라인 먹매김 및 구배 계획, STEP 2: 주철관/PVC관 포설 및 배관 행거 고정 절차서 준수 시공</t>
+          <t>1) STEP 1 (자연유하 구배 시공): 레이저 레벨기를 이용하여 오수관 1/100, 배수관 1/50 구배를 철저히 유지하며 배관 포설
+2) STEP 2 (수중펌프 자동교번 안착): 집수조 바닥에 상용 및 예비 수중펌프 2대를 자동탈착 가이드레일 방식으로 거치
+3) STEP 3 (4단 전극봉 수위 인터록): 정지(LWL), 교번기동(HWL), 동시기동(E-HWL), 고수위경보(Alarm) 4단 센서 작동 검증</t>
         </is>
       </c>
       <c r="L23" s="163" t="inlineStr">
@@ -13183,7 +13227,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="36" customHeight="1" s="147">
+    <row r="24" ht="48" customHeight="1" s="147">
       <c r="A24" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13231,12 +13275,14 @@
       </c>
       <c r="J24" s="156" t="inlineStr">
         <is>
-          <t>차량기지 중정비 공장(대차도장, 대차세척, 부품세척 등 23.314 ㎥/일), 경정비 공장(4.054 ㎥/일) 및 청소선에서 발생하는 고농도 유기계·유류 폐수를 법정 환경 기준 이하로 정화 배출하기 위해 기지 외곽에 연면적 90㎡ 규모의 전용 가설 폐수처리장, 유수분리기, 화학응집침전조 및 활성탄 흡착탑을 완벽 시공한다.</t>
+          <t>중정비·경정비 발생 오폐수(35㎥/일)의 유수분리, 화학응집, 활성탄 흡착 및 수질 TMS 원격 방류</t>
         </is>
       </c>
       <c r="K24" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 폐수처리장(90㎡) 토목 구조물 및 방수 검측, STEP 2: 유수분리기 및 원수 수집조 설비 설치 절차서 준수 시공</t>
+          <t>1) STEP 1 (유수분리기 설치): 차량 정비 폐수의 비중차 유분 분리조 및 오일 스키머 설치로 유분 농도 90% 이상 제거
+2) STEP 2 (응집 침전 및 가압부상): PAC 응집제 및 폴리머 자동 주입기를 통해 플록(Floc) 침전 및 슬러지 탈수기 케이크 처리
+3) STEP 3 (활성탄 흡착 및 TMS 연동): 2단 활성탄 흡착탑 정화 후 BOD/COD ≤ 20mg/L 수질 TMS 데이터 환경청 자동 전송</t>
         </is>
       </c>
       <c r="L24" s="156" t="inlineStr">
@@ -13295,7 +13341,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="36" customHeight="1" s="147">
+    <row r="25" ht="48" customHeight="1" s="147">
       <c r="A25" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13343,12 +13389,14 @@
       </c>
       <c r="J25" s="163" t="inlineStr">
         <is>
-          <t>동탄트램 차량의 청결 상태를 유지하기 위해 차량기지 청소선에 트램 전용 갠트리식 자동세척설비(차체 전·측·후면 브러시, 세제 분사 펌프, 린스 노즐, 윈드 블로워 송풍 건조기, 폐수 회수 집수 트렌치)를 시공하고, 열차 진입 감지 센서 연동 100% 자동 세척 시퀀스를 완성한다.</t>
+          <t>트램 전동차 청소선 세차 갠트리, EVA 무스크래치 브러시 및 세척수 85% 회수 재활용</t>
         </is>
       </c>
       <c r="K25" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 청소선 궤도 건축한계 대조 및 기초 앵커 시공, STEP 2: 세차기 메인 갠트리 프레임 및 브러시 조립 절차서 준수 시공</t>
+          <t>1) STEP 1 (세차 갠트리 프레임 가설): 청소선 궤도 상부에 고압 노즐 파이프 및 갠트리 구조물 용접 앵커링
+2) STEP 2 (EVA 브러시 및 약품 분사): 전동차 차체 도장 손상을 방지하는 초미세 발포 EVA 브러시 및 중성 세제 분사 노즐 세팅
+3) STEP 3 (세척수 회수 트렌치 통수): 하부 STS 그레이팅 트렌치를 통해 세척수 85% 이상 회수 및 순환 정화조 인입 검측</t>
         </is>
       </c>
       <c r="L25" s="163" t="inlineStr">
@@ -13407,7 +13455,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="36" customHeight="1" s="147">
+    <row r="26" ht="48" customHeight="1" s="147">
       <c r="A26" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13455,12 +13503,14 @@
       </c>
       <c r="J26" s="156" t="inlineStr">
         <is>
-          <t>차량기지 종합관리동 및 정거장 정화조 수조에서 발생하는 황화수소(H2S), 암모니아(NH3), 메탄(CH4) 등 유해·악취 가스가 지상 역사 및 근무 공간으로 확산되는 것을 원천 차단하기 위해, 정화조실 내부를 3종 음압으로 유지하는 내식성 FRP 탈취 덕트, 약액세정식 2단 탈취탑 및 복합가스 감지 센서를 시공한다.</t>
+          <t>정화조실 3종 음압(-20Pa) 유지 및 2단 약액세정탑(산/알칼리)+첨착활성탄 복합 탈취</t>
         </is>
       </c>
       <c r="K26" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 정화조실 음압 환기량 및 유해가스 농도 계산, STEP 2: 내식성 FRP 탈취 덕트 및 배기팬 가설 절차서 준수 시공</t>
+          <t>1) STEP 1 (음압 덕트 및 후드 설치): 정화조 발생원 상부에 내식성 FRP 배기 후드 및 전용 음압 배기팬(15~20회/h) 가설
+2) STEP 2 (2단 스크러버 약액 세정): 산(H2SO4) 및 알칼리(NaOH) 세정탑 순환 펌프와 노즐을 통해 황화수소(H2S) 99% 중화
+3) STEP 3 (첨착 활성탄 흡착 배출): 최종 첨착 활성탄 흡착탑을 거쳐 복합악취 희석배수 ≤ 500 이하 기준 충족 확인</t>
         </is>
       </c>
       <c r="L26" s="156" t="inlineStr">
@@ -13519,7 +13569,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="36" customHeight="1" s="147">
+    <row r="27" ht="48" customHeight="1" s="147">
       <c r="A27" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13567,12 +13617,14 @@
       </c>
       <c r="J27" s="163" t="inlineStr">
         <is>
-          <t>화재안전기술기준(NFTC 102) 및 시방서 개선 사항에 따라 일반인이 혼자서도 손쉽게 당겨서 방수할 수 있는 고성능 '호스릴 옥내소화전(STS304 외함, 25mm 고무호스 릴, 분말소화기 3.3kg 2대 내장형)'을 정거장 및 차량기지 전 구역에 보행거리 25m 이내로 배치하고, 방수압력(0.17~0.7MPa) 및 방수량(130L/min)을 완벽 시공한다.</t>
+          <t>STS304 호스릴 옥내소화전(보행거리 25m 이내, 방수압 0.17~0.7MPa) 1인 조작 화재 진압</t>
         </is>
       </c>
       <c r="K27" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 소화전함 설치 위치 먹매김 및 배관 인입선 실측, STEP 2: 배관 가설 및 그루브 조인트(Grooved Joint) 체결 절차서 준수 시공</t>
+          <t>1) STEP 1 (STS304 소화전함 매립): 정거장 및 역사 벽체에 STS304 방청 소화전함을 수직·수평 정밀 매립
+2) STEP 2 (25m 호스릴 및 밸브 체결): 1인 전개 인장력 5kgf 이하의 원형 회전 드럼식 25m 경량 호스릴 및 감압 앵글밸브 설치
+3) STEP 3 (방수압력 및 방수량 실측): 피토게이지를 이용하여 노즐 방수압 0.17~0.7MPa 및 방수량 ≥ 130L/min 20분간 방수 실측</t>
         </is>
       </c>
       <c r="L27" s="163" t="inlineStr">
@@ -13631,7 +13683,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="36" customHeight="1" s="147">
+    <row r="28" ht="48" customHeight="1" s="147">
       <c r="A28" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13679,12 +13731,14 @@
       </c>
       <c r="J28" s="156" t="inlineStr">
         <is>
-          <t>화재안전기술기준(NFTC 103, 502) 개정 법령에 따라 과거 겸용으로 시공되던 '연결송수관설비'와 '스프링클러설비'의 수직 주배관 및 옥외 소방차 연결 송수구를 물리적으로 각각 100% 완전 분리 시공하여, 화재 시 소방차 고압 가압에 따른 스프링클러 배관 파손을 막고 소화 수압 안정성을 극대화한다.</t>
+          <t>개정 화재안전기준에 따른 연결송수관과 스프링클러설비의 주배관 및 옥외 송수구 완전 물리적 분리</t>
         </is>
       </c>
       <c r="K28" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 개정 화재안전기술기준 설계도서 대조 및 입상 경로 분리, STEP 2: 연결송수관 전용 고압 배관 시공 절차서 준수 시공</t>
+          <t>1) STEP 1 (독립 배관 라인 포설): 연결송수관(고압 Sch40)과 스프링클러 알람밸브 2차측 배관을 완전 독립 경로로 가설
+2) STEP 2 (쌍구형 송수구 분리 설치): 옥외 소방차 진입로에 연결송수관용 및 스프링클러용 쌍구형 송수구를 명판과 함께 분리 취부
+3) STEP 3 (2.0MPa 고압 내압시험): 소방차 직결 가압을 상정하여 2.0MPa 압력으로 30분간 내압시험을 실시해 관로 안전성 입증</t>
         </is>
       </c>
       <c r="L28" s="156" t="inlineStr">
@@ -13743,7 +13797,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1" s="147">
+    <row r="29" ht="48" customHeight="1" s="147">
       <c r="A29" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13791,12 +13845,14 @@
       </c>
       <c r="J29" s="163" t="inlineStr">
         <is>
-          <t>전기 스파크 및 과부하로 인한 전기화재 위험이 높은 차량기지 변전소, 트램 배터리 충전 전기실, 종합관리동 및 본선 31개소 정거장의 특고압/저압 수배전반 큐비클(Cubicle) 내부에 KFI 형식승인을 득한 소공간용 고체에어로졸 자동소화장치를 1:1 취부하여 판넬 내부 화재를 3초 이내에 국부 진압한다.</t>
+          <t>특고압/저압 수배전반 판넬 내부 KFI 인증 소공간 고체에어로졸 설치 및 3초 내 초기 진압</t>
         </is>
       </c>
       <c r="K29" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 수배전반 큐비클 체적(㎥) 및 소화약제량 산정, STEP 2: 고체에어로졸 소화장치 브라켓 고정 절차서 준수 시공</t>
+          <t>1) STEP 1 (큐비클 내부 브래킷 고정): 수배전반 상단 발화 예상 지점에 내진 브래킷을 이용하여 에어로졸 소화장치 취부
+2) STEP 2 (열감지선 및 기폭선 결선): 105℃ 정온식 열감지선을 판넬 내부 주요 부스바 주변에 포설하고 제어부 결선
+3) STEP 3 (ACB 차단기 인터록 연동): 화재 감지 및 소화기 기폭 신호 출력 즉시 주차단기(ACB)가 자동 트립되는 인터록 검증</t>
         </is>
       </c>
       <c r="L29" s="163" t="inlineStr">
@@ -13855,7 +13911,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1" s="147">
+    <row r="30" ht="48" customHeight="1" s="147">
       <c r="A30" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -13903,12 +13959,14 @@
       </c>
       <c r="J30" s="156" t="inlineStr">
         <is>
-          <t>차량기지 주변전소, 정거장 변전실 등 가스계 소화설비(HFC-125, Novec 1230 등)가 적용된 밀폐 방호구역에 소화가스 방출 시 순간적인 압력 상승으로 인한 방화벽체, 출입문 및 유리창의 파손을 방지하기 위하여, 설정 압력(150~300Pa) 이상에서 자동으로 개방되는 과압배출구(P.R.D, Pressure Relief Damper)를 벽체에 완벽 가설한다.</t>
+          <t>가스소화약제 방출 시 실내 과압(200Pa) 자동 해소 및 자중 폐쇄를 통한 10분 설계농도 유지</t>
         </is>
       </c>
       <c r="K30" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 가스 방출 압력 상승치 및 P.R.D 배출 면적 계산, STEP 2: 방화벽체 개구부 타공 및 STS 프레임 가설 절차서 준수 시공</t>
+          <t>1) STEP 1 (방화벽체 개구부 프레임 취부): 변전실 외벽 또는 복도측 방화벽체에 P.R.D 댐퍼 프레임 수평 매립 고정
+2) STEP 2 (카운터웨이트 개방압 세팅): 실내 압력이 200Pa에 도달할 때 블레이드가 정확히 열리도록 카운터웨이트 추 정밀 교정
+3) STEP 3 (자중 폐쇄 및 기밀도 검측): 압력 해소 후 중력으로 완벽히 닫혀 소화가스 누출(약제 설계농도 10분 유지) 방지 검증</t>
         </is>
       </c>
       <c r="L30" s="156" t="inlineStr">
@@ -13967,7 +14025,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1" s="147">
+    <row r="31" ht="48" customHeight="1" s="147">
       <c r="A31" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -14015,12 +14073,14 @@
       </c>
       <c r="J31" s="163" t="inlineStr">
         <is>
-          <t>화재안전기술기준(NFTC 102, 103)에 따라 정거장 및 차량기지 지하 소방펌프실에 주펌프(전기모터 구동), 보조 충압펌프, 성능시험배관, 압력챔버(또는 전자식 압력스위치), 순환배관 및 릴리프밸브를 가설하고, 3대 필수 성능시험(체절운전 시험, 정격부하 시험, 150% 최대부하 시험)을 완벽 수행한다.</t>
+          <t>소방펌프실 주/충압펌프 거치 및 체절압력(≤140%), 정격(100%), 150% 부하(≥65%) 법정 성능시험</t>
         </is>
       </c>
       <c r="K31" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 소방펌프 콘크리트 기초 패드 및 방진가대 시공, STEP 2: 흡입·토출 배관, 플렉시블 조인트 및 밸브류 체결 절차서 준수 시공</t>
+          <t>1) STEP 1 (펌프 기초 및 방진가설): 콘크리트 패드 위에 다단원심 소방 주펌프 및 충압펌프 방진마운트 거치 및 축정렬
+2) STEP 2 (성능시험 배관 및 유량계): 주배관에서 분기된 오리피스 차압식 유량계 배관 및 순환배관 릴리프밸브 설치
+3) STEP 3 (3대 법정 성능시험 입회): 감리원 입회 하에 체절운전(정격 140% 이하), 100% 정격부하, 150% 피크부하 곡선 검증</t>
         </is>
       </c>
       <c r="L31" s="163" t="inlineStr">
@@ -14079,7 +14139,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1" s="147">
+    <row r="32" ht="48" customHeight="1" s="147">
       <c r="A32" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -14127,12 +14187,14 @@
       </c>
       <c r="J32" s="156" t="inlineStr">
         <is>
-          <t>교통약자의 수직 이동권 및 환승 편의를 보장하기 위해 정거장 외부 환승 동선에 17인승/24인승 MRL(기계실 없는) 인승용 엘리베이터를 설치하고, 승강로 수직도(±5mm), 가이드레일 브라켓, 도어 다점 적외선 안전센서, 비상통화장치 및 한국승강기안전공단 완성검사를 100% 합격 완료한다.</t>
+          <t>정거장 MRL(기계실 없는) 인승용 승강기 설치 및 KoELSA 완성검사 필증 획득</t>
         </is>
       </c>
       <c r="K32" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 승강로 골조 치수, 피트 깊이 및 수직도 실측, STEP 2: 가이드레일 브라켓 및 T형 레일 조립 절차서 준수 시공</t>
+          <t>1) STEP 1 (승강로 수직도 및 레일 조립): 승강로 수직도(오차 ≤ ±5mm) 실측 후 13K 가이드레일 브래킷 앵커링 및 조립
+2) STEP 2 (PMSM 권상기 및 카 조립): PMSM 영구자석 기어리스 권상기 안착, 메인로프(안전율 ≥ 12) 텐션 조정 및 카 조립
+3) STEP 3 (KoELSA 법정 완성검사): 128채널 3D 도어센서, 정전 시 ARD 구출장치, 조속기 비상정지장치 실부하 시험 100% 합격</t>
         </is>
       </c>
       <c r="L32" s="156" t="inlineStr">
@@ -14191,7 +14253,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="36" customHeight="1" s="147">
+    <row r="33" ht="48" customHeight="1" s="147">
       <c r="A33" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -14239,12 +14301,14 @@
       </c>
       <c r="J33" s="163" t="inlineStr">
         <is>
-          <t>차량기지 종합검수고동 내 무거운 트램 부품, 대차 예비품 및 정비 공구의 층간 수직 이동을 전담하기 위해 3~5ton급 대용량 '관통형(양방향 도어 개폐형) 화물용 엘리베이터'를 설치하고, 지게차 진입 충격에 견디는 바닥 하중 보강, 도어 씰(Sill) 보강 및 화물 전용 안전장치를 완벽 시공한다.</t>
+          <t>차량기지 종합검수고 관통형(양방향 도어) 3~5ton 화물용 승강기 가설 및 지게차 진입 바닥 보강</t>
         </is>
       </c>
       <c r="K33" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 대형 화물용 승강로 구조 및 지게차 동선 검토, STEP 2: 대형 H형강 카 프레임 및 중량 레일 가설 절차서 준수 시공</t>
+          <t>1) STEP 1 (중하중 승강로 구조 보강): 지게차(자중 4.5ton) 진입 하중을 견디도록 카 바닥 H형강 및 4.5T 체크플레이트 보강
+2) STEP 2 (관통형 양방향 도어 인터록): 1층 전면 도어와 2층 후면 도어가 동시 개방되지 않도록 안전 인터록 릴레이 구축
+3) STEP 3 (125% 과부하 하중시험): 정격 적재하중의 125%(6.25ton) 추를 탑재하여 권상 제동력 및 슬립 유무 정밀 안전검사</t>
         </is>
       </c>
       <c r="L33" s="163" t="inlineStr">
@@ -14303,7 +14367,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="36" customHeight="1" s="147">
+    <row r="34" ht="48" customHeight="1" s="147">
       <c r="A34" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -14351,12 +14415,14 @@
       </c>
       <c r="J34" s="156" t="inlineStr">
         <is>
-          <t>정거장 및 차량기지 내 모든 기계설비(공조기, 환기팬, 펌프, 댐퍼, 밸브, 저수조, 전력계)의 실시간 원격 감시 및 에너지 최적 제어를 위해 직접디지털제어(DDC/IP DDC) 패널을 가설하고, 개방형 BACnet/Modbus 프로토콜 적용 및 메인 서버 장애 시 0초 무중단 자동 절환되는 Backup Server 이중화 시스템을 완벽 구축한다.</t>
+          <t>기계설비 직접디지털제어(IP DDC) 판넬 설치, BACnet 국제표준 통신 및 관제서버 무중단 이중화</t>
         </is>
       </c>
       <c r="K34" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 자동제어 I/O 포인트 일람표 및 통신 선로 설계 대조, STEP 2: 기계실 IP DDC 패널 가설 및 필드 센서/밸브 배선 절차서 준수 시공</t>
+          <t>1) STEP 1 (IP DDC 필드 제어반 결선): 기계실 및 공조실 DDC 판넬에 아날로그(AI/AO), 디지털(DI/DO) 센서·밸브 케이블 결선
+2) STEP 2 (BACnet 통신 루프 구축): 개방형 BACnet/IP 프로토콜을 적용하여 중앙 방재실 관제 컴퓨터와 실시간 데이터 통신 연동
+3) STEP 3 (서버 0초 이중화 절환 시험): 메인 관제 서버 강제 다운 시 대기 중인 백업 서버로 데이터 손실 없이 0초 절환 검증</t>
         </is>
       </c>
       <c r="L34" s="156" t="inlineStr">
@@ -14415,7 +14481,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="36" customHeight="1" s="147">
+    <row r="35" ht="48" customHeight="1" s="147">
       <c r="A35" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -14463,12 +14529,14 @@
       </c>
       <c r="J35" s="163" t="inlineStr">
         <is>
-          <t>화재안전기술기준 및 철도 방재 매뉴얼에 따라 화재 발생 시 연기가 공조 덕트를 타고 다른 구역으로 확산되는 대형 참사를 막기 위해, 화재수신반 경보 발생 즉시 공조기·냉난방기 마그네틱 전원을 100% 강제 차단하고, 해당 제연구역의 제연팬을 비상 배연 모드로 가동하는 방재 인터록 실부하 시험을 수행한다.</t>
+          <t>화재 수신반 신호 수신 즉시 공조기 100% 강제 정지 및 제연팬 배연 모드 자동 인터록</t>
         </is>
       </c>
       <c r="K35" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 화재 연동 방재 매트릭스(Cause &amp; Effect) 수립, STEP 2: 공조기 MCC 정지 접점 및 제연팬 기동 결선 점검 절차서 준수 시공</t>
+          <t>1) STEP 1 (하드와이어드 인터록 회로 구성): 화재수신반 경보 접점을 공조기 MCC 조작전원 차단 계전기(B접점)와 직결
+2) STEP 2 (제연댐퍼 및 팬 시퀀스 연동): 화재 구역 제연 풍도 댐퍼가 완전 개방된 후 리미트 스위치 신호로 제연팬 자동 가동
+3) STEP 3 (실부하 화재 모의시험): 연기감지기 실발화 시험을 실시하여 3초 이내 공조기 정지 및 제연팬 정상 기동 확인</t>
         </is>
       </c>
       <c r="L35" s="163" t="inlineStr">
@@ -14527,7 +14595,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="36" customHeight="1" s="147">
+    <row r="36" ht="48" customHeight="1" s="147">
       <c r="A36" s="153" t="inlineStr">
         <is>
           <t>9000</t>
@@ -14575,12 +14643,14 @@
       </c>
       <c r="J36" s="156" t="inlineStr">
         <is>
-          <t>공조 및 배관 시스템의 완성도를 입증하고 실내 쾌적 환경과 에너지를 최적화하기 위해, 국가공인 TAB(Testing, Adjusting, Balancing) 전문기관에 의뢰하여 정거장 및 차량기지 전 구역의 공조 덕트 풍량, 디퓨저 취출 기류, 냉온수 배관 유량 및 실내 소음·차압을 정밀 측정하고 설계치 대비 오차 ±10% 이내로 균일 밸런싱한다.</t>
+          <t>공조 덕트 풍량(오차 ±10% 이내) 및 수배관 유량 정밀 측정·조정(TAB)으로 쾌적성 확보</t>
         </is>
       </c>
       <c r="K36" s="156" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: TAB 사전 검토 및 측정 계획서 수립, STEP 2: 공조 덕트 주풍량 및 디퓨저 풍량 측정·조정 절차서 준수 시공</t>
+          <t>1) STEP 1 (공조 덕트 풍량 TAB): 피토관 및 플로우 후드를 이용하여 주덕트와 각 디퓨저 취출 풍량을 설계치 ±10%로 교정
+2) STEP 2 (수배관 유량 TAB): 초음파 비파괴 유량계로 냉온수 배관 순환 유량을 측정하고 밸런싱 밸브 차압(ΔP) 정밀 조정
+3) STEP 3 (소음 및 온습도 검증): 정거장 실내 소음(NC 35~40) 및 실별 온·습도 분포도를 24시간 연속 측정하여 TAB 성적서 발급</t>
         </is>
       </c>
       <c r="L36" s="156" t="inlineStr">
@@ -14639,7 +14709,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="36" customHeight="1" s="147">
+    <row r="37" ht="48" customHeight="1" s="147">
       <c r="A37" s="160" t="inlineStr">
         <is>
           <t>9000</t>
@@ -14687,12 +14757,14 @@
       </c>
       <c r="J37" s="163" t="inlineStr">
         <is>
-          <t>동탄트램 기계설비 및 소방공사의 최종 마무리를 위해 관할 소방서(화성소방서 등)의 엄격한 현장 실사를 통해 '소방시설 완공검사증명서(소방필증)'를 획득하고, 준공도면(As-Built), 장비 매뉴얼, 예비품 목록, 종합시운전 성적서를 완비하여 화성도시공사 기계·소방 운영유지관리팀에 무결점 종합 인수인계를 완료한다.</t>
+          <t>관할 소방서 완공검사필증 획득, As-Built 준공도서 편찬 및 운영사(화성도시공사) 무결점 인수인계</t>
         </is>
       </c>
       <c r="K37" s="163" t="inlineStr">
         <is>
-          <t>KCS 41 시방 기준 및 STEP 1: 소방시설 완공검사 신청서 제출 및 사전 자체 점검, STEP 2: 관할 소방서 합동 현장 실사 및 성능 시연 절차서 준수 시공</t>
+          <t>1) STEP 1 (관할 소방서 완공 실사): 소방감리원 및 소방관 합동 현장 실사를 통해 소화·경보·피난설비 전수 작동 검사
+2) STEP 2 (소방완공검사필증 수령): 지적사항 0건으로 소방시설 완공검사증명서(필증)를 정식 교부받아 법적 준공 완료
+3) STEP 3 (준공도서 및 운영자 교육): 3D As-Built 준공도면, 시운전 성적서, 2년분 예비품을 인계하고 운영팀 40시간 기술교육 이수</t>
         </is>
       </c>
       <c r="L37" s="163" t="inlineStr">

</xml_diff>